<commit_message>
refactor: enhance rule similarity scoring and update spreadsheet loading logic
</commit_message>
<xml_diff>
--- a/extracoes_manuais_validadas.xlsx
+++ b/extracoes_manuais_validadas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Id_arquivo</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>Regras formatadas e validadas</t>
+  </si>
+  <si>
+    <t>01</t>
   </si>
   <si>
     <t>01_documento_orientador_emissao_de_diploma-ensino_medio-ifba</t>
@@ -104,6 +107,9 @@
       "referencia": "Item 2.7"
     }
   ]</t>
+  </si>
+  <si>
+    <t>02</t>
   </si>
   <si>
     <t>02_Edital_n_C2_BA_13_2024_Estagio_versao_final_assina_240905_230648</t>
@@ -198,6 +204,9 @@
       "referencia": "Item 3.2.2"
     }
   ]</t>
+  </si>
+  <si>
+    <t>10</t>
   </si>
   <si>
     <t>EDITAL DE APOIO A CONCESSÃO DE DIÁRIAS E PASSAGENS</t>
@@ -325,6 +334,9 @@
       "referencia": "Item 2.6"
     }
   ]</t>
+  </si>
+  <si>
+    <t>28</t>
   </si>
   <si>
     <t>Edital_N_C2_BA_13.2025.DG.DEMAT.IFA_SSA_assinado__1_</t>
@@ -592,7 +604,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -611,8 +623,8 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
@@ -628,6 +640,9 @@
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -977,20 +992,20 @@
       <c r="W1" s="5"/>
     </row>
     <row r="2" ht="216.75" customHeight="1">
-      <c r="A2" s="6">
-        <v>1.0</v>
+      <c r="A2" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1011,18 +1026,18 @@
       <c r="W2" s="11"/>
     </row>
     <row r="3" ht="382.5" customHeight="1">
-      <c r="A3" s="6">
-        <v>2.0</v>
+      <c r="A3" s="6" t="s">
+        <v>10</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="11"/>
@@ -1044,18 +1059,18 @@
       <c r="W3" s="11"/>
     </row>
     <row r="4" ht="558.0" customHeight="1">
-      <c r="A4" s="6">
-        <v>10.0</v>
+      <c r="A4" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>16</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="11"/>
@@ -1077,37 +1092,37 @@
       <c r="W4" s="11"/>
     </row>
     <row r="5" ht="807.0" customHeight="1">
-      <c r="A5" s="6">
-        <v>28.0</v>
+      <c r="A5" s="12" t="s">
+        <v>18</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F5" s="7"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="14"/>
+      <c r="U5" s="14"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="14"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
feat: implement batch processing for document extraction and update evaluation metrics
</commit_message>
<xml_diff>
--- a/extracoes_manuais_validadas.xlsx
+++ b/extracoes_manuais_validadas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Id_arquivo</t>
   </si>
@@ -561,6 +561,287 @@
       "referencia": "Item 8.1.1 (b)"
     }
   ]</t>
+  </si>
+  <si>
+    <t>RESOLUÇÃO Nº 32, DE 09 DE OUTUBRO DE 2018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Art. 7º Os representantes docentes e técnico-administrativos eleitos por seus pares não poderão:
+I. estar no exercício de cargo de direção (CD);
+II. estar afastado para qualificação;
+III. ser membro titular ou suplente do Conselho Superior (CONSUP);
+IV. ser membro da Comissão Própria de Avaliação (CPA);
+V. ser membro da Comissão Permanente Pessoal Docente (CPPD); ou
+VI. ser membro da Comissão Interna de Supervisão do Plano de Cargos e Carreira dos TécnicosAdministrativos em Educação (CIS/PCCTAE).
+Art. 9º Os representantes do Conselho de cada Campus não poderão:
+I. estar afastado para qualificação;
+II. ser membro titular ou suplente do Conselho Superior (CONSUP);
+III. ser membro da Comissão Própria de Avaliação (CPA);
+IV. ser membro da Comissão Permanente Pessoal Docente (CPPD);
+V. ser membro da Comissão Interna de Supervisão do Plano de Cargos e Carreira dos TécnicosAdministrativos em Educação (CIS/PCCTAE); ou
+VI. ser membro do Colégio de Dirigentes.
+Art. 10. Os representantes discentes e seus respectivos suplentes deverão ter matrícula regular ativa nos
+cursos de educação profissional técnica de nível médio e/ou de educação superior de graduação e pósgraduação, independentemente da modalidade, conforme distribuição expressa no inciso VIII, do Artigo 2º.
+Art. 11. Os representantes titulares e suplentes dos discentes não poderão:
+I. ter matrícula trancada;
+II. ser membro titular ou suplente do Conselho Superior (CONSUP); ou
+III. ser membro da Comissão Própria de Avaliação (CPA).
+§ 4º O membro do Conselho que, por motivo justificado, não puder comparecer a uma reunião, deverá
+comunicar o fato à secretaria num prazo de até 48 (quarenta e oito) horas de antecedência da reunião.
+§ 1º O processo recebido com pedido de vista deve ser devolvido em até 10 (dez) dias úteis após a data da
+reunião, vedado novo pedido, salvo se autorizado pelo Presidente do Conselho.
+§ 2º O processo do qual foi pedido vista deve retornar ao seu relator.
+Art. 44. A apreciação das matérias constantes da pauta deve atender aos seguintes procedimentos:
+I. apresentação da matéria pelo Presidente;
+II. leitura do parecer;
+III. discussão da matéria e do parecer, mediante concessão da palavra aos membros, pela ordem de sua
+inscrição;
+IV. síntese das propostas, com enumeração por escrito das propostas apresentadas durante a discussão;
+V. votação da matéria;
+VI. encaminhamentos.
+Art. 51. Os pareceres ou deliberações emanadas das câmaras e comissões devem ser submetidos ao
+CONSEPE para análise, deliberação e/ou homologação.
+</t>
+  </si>
+  <si>
+    <t>"regras": [
+    {
+    "id": "R01",
+    "descricao": "Não estar no exercício de cargo de direção (CD).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — I"
+    },
+    {
+    "id": "R02",
+    "descricao": "Não estar afastado para qualificação.",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — II"
+    },
+    {
+    "id": "R03",
+    "descricao": "Não ser membro titular ou suplente do Conselho Superior (CONSUP).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — III"
+    },
+    {
+    "id": "R04",
+    "descricao": "Não ser membro da Comissão Própria de Avaliação (CPA).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — IV"
+    },
+    {
+    "id": "R05",
+    "descricao": "Não ser membro da Comissão Permanente Pessoal Docente (CPPD).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — V"
+    },
+    {
+    "id": "R06",
+    "descricao": "Não ser membro da Comissão Interna de Supervisão do Plano de Cargos e Carreira dos Técnicos-Administrativos em Educação (CIS/PCCTAE).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes docentes e técnico-administrativos eleitos por seus pares.",
+    "referencia": "Art. 7º — VI"
+    },
+    {
+    "id": "R07",
+    "descricao": "Não estar afastado para qualificação.",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — I"
+    },
+    {
+    "id": "R08",
+    "descricao": "Não ser membro titular ou suplente do Conselho Superior (CONSUP).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — II"
+    },
+    {
+    "id": "R09",
+    "descricao": "Não ser membro da Comissão Própria de Avaliação (CPA).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — III"
+    },
+    {
+    "id": "R10",
+    "descricao": "Não ser membro da Comissão Permanente Pessoal Docente (CPPD).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — IV"
+    },
+    {
+    "id": "R11",
+    "descricao": "Não ser membro da Comissão Interna de Supervisão do Plano de Cargos e Carreira dos Técnicos-Administrativos em Educação (CIS/PCCTAE).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — V"
+    },
+    {
+    "id": "R12",
+    "descricao": "Não ser membro do Colégio de Dirigentes.",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes do Conselho de cada Campus.",
+    "referencia": "Art. 9º — VI"
+    },
+    {
+    "id": "R13",
+    "descricao": "Ter matrícula regular ativa nos cursos de educação profissional técnica de nível médio e/ou de educação superior de graduação e pós-graduação.",
+    "tipo": "obrigatória",
+    "condicao": "Apenas para representantes discentes e seus respectivos suplentes.",
+    "referencia": "Art. 10"
+    },
+    {
+    "id": "R14",
+    "descricao": "Não ter matrícula trancada.",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes titulares e suplentes dos discentes.",
+    "referencia": "Art. 11 — I"
+    },
+    {
+    "id": "R15",
+    "descricao": "Não ser membro titular ou suplente do Conselho Superior (CONSUP).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes titulares e suplentes dos discentes.",
+    "referencia": "Art. 11 — II"
+    },
+    {
+    "id": "R16",
+    "descricao": "Não ser membro da Comissão Própria de Avaliação (CPA).",
+    "tipo": "restritiva",
+    "condicao": "Apenas para representantes titulares e suplentes dos discentes.",
+    "referencia": "Art. 11 — III"
+    },
+    {
+    "id": "R17",
+    "descricao": "Comunicar o fato à secretaria num prazo de até 48 horas de antecedência da reunião.",
+    "tipo": "condicional",
+    "condicao": "Caso o membro do Conselho não puder comparecer a uma reunião por motivo justificado.",
+    "referencia": "§ 4º"
+    },
+    {
+    "id": "R18",
+    "descricao": "Devolver o processo recebido com pedido de vista em até 10 dias úteis após a data da reunião.",
+    "tipo": "obrigatória",
+    "condicao": null,
+    "referencia": "§ 1º"
+    },
+    {
+    "id": "R19",
+    "descricao": "Não realizar novo pedido de vista no mesmo processo.",
+    "tipo": "restritiva",
+    "condicao": "Salvo se expressamente autorizado pelo Presidente do Conselho.",
+    "referencia": "§ 1º"
+    },
+    {
+    "id": "R20",
+    "descricao": "Retornar o processo do qual foi pedido vista ao seu relator.",
+    "tipo": "obrigatória",
+    "condicao": null,
+    "referencia": "§ 2º"
+    },
+    {
+    "id": "R21",
+    "descricao": "Atender aos seguintes procedimentos na apreciação das matérias: apresentação pelo Presidente, leitura do parecer, discussão mediante inscrição, síntese escrita das propostas, votação e encaminhamentos.",
+    "tipo": "obrigatória",
+    "condicao": null,
+    "referencia": "Art. 44 — I a VI"
+    },
+    {
+    "id": "R22",
+    "descricao": "Submeter os pareceres ou deliberações emanadas das câmaras e comissões ao CONSEPE para análise, deliberação e/ou homologação.",
+    "tipo": "obrigatória",
+    "condicao": null,
+    "referencia": "Art. 51"
+    }
+]</t>
+  </si>
+  <si>
+    <t>INGRESSO 2026.2 - SIMPLIFICADO SUBSEQUENTE 2026.2 - 2026.2 SUBSEQUENTE INGRESSO SIMPLIFICADO</t>
+  </si>
+  <si>
+    <t>4.11 Para realizar corretamente sua inscrição e concorrer ao Ingresso Simplificado 2026.2, a pessoa candidata
+deverá realizar os seguintes PASSOS, conforme indicados pelo sistema de inscrição:
+I. Acessar o sistema online de inscrições do Ingresso Simplificado 2026.2 disponível no link:
+https://portal.ifba.edu.br/proen/2026/simplificadosub/2 ;
+II. Criar seu cadastro no sistema (caso ainda não tenha), informando o número de CPF da própria pessoa
+candidata e criando uma senha pessoal;
+III. Informar todos os dados pessoais solicitados da pessoa candidata;
+IV. Informar a escolaridade e tipos de escola (se pública ou privada) em que a pessoa candidata cursou
+todo o Ensino Médio (incluso 3º ano em curso, se for o caso).
+V. ESCOLHER O CAMPUS ONDE DESEJA ESTUDAR;
+VI. Selecionar um curso para o qual deseja se inscrever como 1ª opção;
+VII. Selecionar um curso diferente para se inscrever como 2ª opção, (caso o campus disponha de mais de
+um curso na mesma forma de oferta);
+VIII. Escolher o tipo de vaga que deseja concorrer, se por reservas de vagas (cotas) ou Ampla
+Concorrência, observando se atende aos critérios para cada tipo de vaga.</t>
+  </si>
+  <si>
+    <t>{
+  "regras": [
+    {
+      "id": "R01",
+      "descricao": "Acessar o sistema online de inscrições do Ingresso Simplificado 2026.2 disponível no link: https://portal.ifba.edu.br/proen/2026/simplificadosub/2.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (I)"
+    },
+    {
+      "id": "R02",
+      "descricao": "Criar seu cadastro no sistema, informando o número de CPF da própria pessoa candidata e criando uma senha pessoal.",
+      "tipo": "condicional",
+      "condicao": "Caso a pessoa candidata ainda não tenha cadastro no sistema.",
+      "referencia": "Item 4.11 (II)"
+    },
+    {
+      "id": "R03",
+      "descricao": "Informar todos os dados pessoais solicitados da pessoa candidata.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (III)"
+    },
+    {
+      "id": "R04",
+      "descricao": "Informar a escolaridade e tipos de escola (se pública ou privada) em que a pessoa candidata cursou todo o Ensino Médio (incluso 3º ano em curso, se for o caso).",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (IV)"
+    },
+    {
+      "id": "R05",
+      "descricao": "Escolher o campus onde deseja estudar.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (V)"
+    },
+    {
+      "id": "R06",
+      "descricao": "Selecionar um curso para o qual deseja se inscrever como 1ª opção.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (VI)"
+    },
+    {
+      "id": "R07",
+      "descricao": "Selecionar um curso diferente para se inscrever como 2ª opção.",
+      "tipo": "condicional",
+      "condicao": "Caso o campus escolhido disponha de mais de um curso na mesma forma de oferta.",
+      "referencia": "Item 4.11 (VII)"
+    },
+    {
+      "id": "R08",
+      "descricao": "Escolher o tipo de vaga que deseja concorrer, se por reservas de vagas (cotas) ou Ampla Concorrência, observando se atende aos critérios para cada tipo de vaga.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 4.11 (VIII)"
+    }
+  ]
+}</t>
   </si>
 </sst>
 </file>
@@ -712,7 +993,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A5:W5" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A5:W7" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="23">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -950,7 +1231,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="11.38"/>
     <col customWidth="1" min="2" max="2" width="52.75"/>
-    <col customWidth="1" min="3" max="3" width="70.75"/>
+    <col customWidth="1" min="3" max="3" width="82.88"/>
     <col customWidth="1" min="4" max="4" width="39.25"/>
     <col customWidth="1" min="5" max="5" width="229.13"/>
     <col customWidth="1" min="6" max="6" width="28.75"/>
@@ -1124,6 +1405,72 @@
       <c r="V5" s="14"/>
       <c r="W5" s="14"/>
     </row>
+    <row r="6" ht="513.75" customHeight="1">
+      <c r="A6" s="12">
+        <v>36.0</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+    </row>
+    <row r="7" ht="396.0" customHeight="1">
+      <c r="A7" s="12">
+        <v>41.0</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="9"/>
+      <c r="E7" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: enhance pipeline configuration and batch processing parameters
</commit_message>
<xml_diff>
--- a/extracoes_manuais_validadas.xlsx
+++ b/extracoes_manuais_validadas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Id_arquivo</t>
   </si>
@@ -334,6 +334,49 @@
       "referencia": "Item 2.6"
     }
   ]</t>
+  </si>
+  <si>
+    <t>Resolucao-N-1110-2015-afastamento-pos-graduacao</t>
+  </si>
+  <si>
+    <t>a) comprovante de aprovação no programa de pós-graduação;
+b) formulário de afastamento, fornecido pela Pró-reitoria de Gestão e Desenvolvimento de Pessoas (PGDP) devidamente preenchido;
+c) termo de compromisso de retorno ao Departamento de lotação; e,
+d) Declaração do Departamento de atendimento ao exposto no Art. 3o desta Resolução.</t>
+  </si>
+  <si>
+    <t>{
+  "regras": [
+    {
+      "id": "R01",
+      "descricao": "Apresentar comprovante de aprovação no programa de pós-graduação.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Alínea a"
+    },
+    {
+      "id": "R02",
+      "descricao": "Apresentar formulário de afastamento, fornecido pela Pró-reitoria de Gestão e Desenvolvimento de Pessoas (PGDP), devidamente preenchido.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Alínea b"
+    },
+    {
+      "id": "R03",
+      "descricao": "Apresentar termo de compromisso de retorno ao Departamento de lotação.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Alínea c"
+    },
+    {
+      "id": "R04",
+      "descricao": "Apresentar Declaração do Departamento de atendimento ao exposto no Art. 3º desta Resolução.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Alínea d"
+    }
+  ]
+}</t>
   </si>
   <si>
     <t>28</t>
@@ -760,6 +803,59 @@
     "referencia": "Art. 51"
     }
 ]</t>
+  </si>
+  <si>
+    <t>edital-no-29-2024-prpgi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1 Serão elegíveis as propostas submetidas pelo responsável pelo Laboratório onde estão as instalações/equipamento multiusuário conforme declaração da direção
+do Campus;
+3.2 O Laboratório e os equipamento deverão estar registrados junto à PRPGI, conforme orientações fornecidas às direções/coordenações de pesquisa dos Campi;
+3.3 O proponente precisa estar adimplente com todos os programas da PRPGI;
+3.4 O proponente deverá pertencer ao quadro de docentes ativos e permantes de um programa de pós-graduação stricto sensu do IFBA;
+3.5 As propostas deverão estar devidamente justificadas quanto a utilização dos recursos no âmbito da pós-graduação.
+</t>
+  </si>
+  <si>
+    <t>{
+  "regras": [
+    {
+      "id": "R01",
+      "descricao": "Submeter a proposta por meio do responsável pelo Laboratório onde estão as instalações/equipamento multiusuário, conforme declaração da direção do Campus.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 3.1"
+    },
+    {
+      "id": "R02",
+      "descricao": "Garantir que o Laboratório e os equipamentos estejam registrados junto à PRPGI, conforme orientações fornecidas às direções/coordenações de pesquisa dos Campi.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 3.2"
+    },
+    {
+      "id": "R03",
+      "descricao": "Estar adimplente com todos os programas da PRPGI.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 3.3"
+    },
+    {
+      "id": "R04",
+      "descricao": "Pertencer ao quadro de docentes ativos e permanentes de um programa de pós-graduação stricto sensu do IFBA.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 3.4"
+    },
+    {
+      "id": "R05",
+      "descricao": "Apresentar propostas devidamente justificadas quanto à utilização dos recursos no âmbito da pós-graduação.",
+      "tipo": "obrigatória",
+      "condicao": null,
+      "referencia": "Item 3.5"
+    }
+  ]
+}</t>
   </si>
   <si>
     <t>INGRESSO 2026.2 - SIMPLIFICADO SUBSEQUENTE 2026.2 - 2026.2 SUBSEQUENTE INGRESSO SIMPLIFICADO</t>
@@ -993,7 +1089,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A5:W7" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A6:W9" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="23">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1372,19 +1468,19 @@
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
     </row>
-    <row r="5" ht="807.0" customHeight="1">
-      <c r="A5" s="12" t="s">
+    <row r="5" ht="396.0" customHeight="1">
+      <c r="A5" s="12">
+        <v>23.0</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>20</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="14"/>
@@ -1405,14 +1501,14 @@
       <c r="V5" s="14"/>
       <c r="W5" s="14"/>
     </row>
-    <row r="6" ht="513.75" customHeight="1">
-      <c r="A6" s="12">
-        <v>36.0</v>
+    <row r="6" ht="807.0" customHeight="1">
+      <c r="A6" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="10" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="9"/>
@@ -1438,14 +1534,14 @@
       <c r="V6" s="14"/>
       <c r="W6" s="14"/>
     </row>
-    <row r="7" ht="396.0" customHeight="1">
+    <row r="7" ht="513.75" customHeight="1">
       <c r="A7" s="12">
-        <v>41.0</v>
+        <v>36.0</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="13" t="s">
         <v>26</v>
       </c>
       <c r="D7" s="9"/>
@@ -1471,6 +1567,72 @@
       <c r="V7" s="14"/>
       <c r="W7" s="14"/>
     </row>
+    <row r="8" ht="396.0" customHeight="1">
+      <c r="A8" s="12">
+        <v>39.0</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="9"/>
+      <c r="E8" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="14"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+    </row>
+    <row r="9" ht="396.0" customHeight="1">
+      <c r="A9" s="12">
+        <v>41.0</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="9"/>
+      <c r="E9" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="14"/>
+      <c r="T9" s="14"/>
+      <c r="U9" s="14"/>
+      <c r="V9" s="14"/>
+      <c r="W9" s="14"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix: exclude '_lotes' from JSON file evaluation in results directory
</commit_message>
<xml_diff>
--- a/extracoes_manuais_validadas.xlsx
+++ b/extracoes_manuais_validadas.xlsx
@@ -345,8 +345,7 @@
 d) Declaração do Departamento de atendimento ao exposto no Art. 3o desta Resolução.</t>
   </si>
   <si>
-    <t>{
-  "regras": [
+    <t xml:space="preserve">  "regras": [
     {
       "id": "R01",
       "descricao": "Apresentar comprovante de aprovação no programa de pós-graduação.",
@@ -376,7 +375,7 @@
       "referencia": "Alínea d"
     }
   ]
-}</t>
+</t>
   </si>
   <si>
     <t>28</t>
@@ -817,8 +816,7 @@
 </t>
   </si>
   <si>
-    <t>{
-  "regras": [
+    <t xml:space="preserve">  "regras": [
     {
       "id": "R01",
       "descricao": "Submeter a proposta por meio do responsável pelo Laboratório onde estão as instalações/equipamento multiusuário, conforme declaração da direção do Campus.",
@@ -854,8 +852,7 @@
       "condicao": null,
       "referencia": "Item 3.5"
     }
-  ]
-}</t>
+  ]</t>
   </si>
   <si>
     <t>INGRESSO 2026.2 - SIMPLIFICADO SUBSEQUENTE 2026.2 - 2026.2 SUBSEQUENTE INGRESSO SIMPLIFICADO</t>
@@ -878,8 +875,7 @@
 Concorrência, observando se atende aos critérios para cada tipo de vaga.</t>
   </si>
   <si>
-    <t>{
-  "regras": [
+    <t xml:space="preserve">  "regras": [
     {
       "id": "R01",
       "descricao": "Acessar o sistema online de inscrições do Ingresso Simplificado 2026.2 disponível no link: https://portal.ifba.edu.br/proen/2026/simplificadosub/2.",
@@ -936,8 +932,7 @@
       "condicao": null,
       "referencia": "Item 4.11 (VIII)"
     }
-  ]
-}</t>
+  ]</t>
   </si>
 </sst>
 </file>

</xml_diff>